<commit_message>
komatsu_can JD CAT D6N E GRADER M_xls
</commit_message>
<xml_diff>
--- a/app/src/main/assets/Komatsu_Can.xlsx
+++ b/app/src/main/assets/Komatsu_Can.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rricotti\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8A5EFA-39A0-4992-A843-5527DE7BDE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF5596F1-8B0B-418D-A964-74042558D951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{FBD1A101-A936-489B-942D-557FED93F0CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FBD1A101-A936-489B-942D-557FED93F0CD}"/>
   </bookViews>
   <sheets>
     <sheet name="KOMATSU CAN" sheetId="1" r:id="rId1"/>
     <sheet name="CAT" sheetId="2" r:id="rId2"/>
+    <sheet name="JOHN DEERE" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="65">
   <si>
     <t>LEICA</t>
   </si>
@@ -181,16 +182,74 @@
   </si>
   <si>
     <t>10=AUTO SIDESHIFT TOGGLE</t>
+  </si>
+  <si>
+    <t>00CF00D80</t>
+  </si>
+  <si>
+    <t>03=AUTO</t>
+  </si>
+  <si>
+    <t>02=MAN</t>
+  </si>
+  <si>
+    <t>12=MAN +OFF</t>
+  </si>
+  <si>
+    <t>22=MAN -OFF</t>
+  </si>
+  <si>
+    <t>13=AUTO +OFF</t>
+  </si>
+  <si>
+    <t>23=AUTO -OFF</t>
+  </si>
+  <si>
+    <t>00EFFF85</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
+    <t>1A</t>
+  </si>
+  <si>
+    <t>4E</t>
+  </si>
+  <si>
+    <t>CONTROL 50MS</t>
+  </si>
+  <si>
+    <t>10000=MAX UP</t>
+  </si>
+  <si>
+    <t>LEFT VALUE 20000=0</t>
+  </si>
+  <si>
+    <t>30000=MAX DW</t>
+  </si>
+  <si>
+    <t>ATTENZIONE AI VALOREI TROPPO LONTANI DA 20.000</t>
+  </si>
+  <si>
+    <t>JD 700L</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -216,11 +275,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -964,4 +1024,197 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B40406C-6026-4A37-851E-C8F4562247BC}">
+  <dimension ref="A1:P20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H3" s="1"/>
+      <c r="L3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="E4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="E5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>